<commit_message>
feat(security): enforce @risel.com.br email domain
Restrict user creation and access to corporate email accounts only across all authentication flows. Also updated the SharePoint sinistros URL and added custom map popup styles.
</commit_message>
<xml_diff>
--- a/data/Comunicado de Sinistro_Frota Pesada.xlsx
+++ b/data/Comunicado de Sinistro_Frota Pesada.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="515" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B22CFC19-56B0-4D70-99CD-230D7FB27B74}"/>
+  <xr:revisionPtr revIDLastSave="519" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE2DE28-8AC7-4A85-AE1E-89255EACDEF1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="77" r:id="rId3"/>
+    <pivotCache cacheId="188" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1873" uniqueCount="1387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1898" uniqueCount="1404">
   <si>
     <t>Id</t>
   </si>
@@ -4188,6 +4188,57 @@
   </si>
   <si>
     <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/FRENTE_Paulo%20Alves%20Pereira%201.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/LATERAL%20DIREITA_Paulo%20Alves%20Pereira%201.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/LATERAL%20ESQUERDA_Paulo%20Alves%20Pereira%201.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/TRASEIRA_Paulo%20Alves%20Pereira%201.jpeg</t>
+  </si>
+  <si>
+    <t>18:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AV LIONS, 2333, PAULICEIA- SÃO BERNARDO DO CAMPO- SP </t>
+  </si>
+  <si>
+    <t>TTB8C36</t>
+  </si>
+  <si>
+    <t>ROBERTO OLIVEIRA DOS SANTOS</t>
+  </si>
+  <si>
+    <t>MILTON ALVES DOS SANTOS</t>
+  </si>
+  <si>
+    <t>11983749050</t>
+  </si>
+  <si>
+    <t>CZW5D96</t>
+  </si>
+  <si>
+    <t>MOTORISTA TENTOU ULTRAPASSAR O FROTA E ENTROU NO PONTO CEGO DO FROTA OCASIONANDO UMA LEVE BATIDA</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/Pergunta/aviso%20de%20sinistro_Camila%20Silva%20Henriqu%201.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/AVISO%20DE%20SINISTRO/registro%20de%20ocorrencia_Camila%20Silva%20Henriqu%201.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA/Boletin%20de%20Ocorr%C3%AAncia%20Roberto%20Oliveira%20Frota_Camila%20Silva%20Henriqu.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DECLARA%C3%87%C3%83O%20DE%20PR%C3%93PRIO%20PUNHO/CNH-e%20ROBERTO%20OLIVEIRA_Camila%20Silva%20Henriqu.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/CNH%20MOTORISTA%20RISEL/F3225%20CRLV%20-%20TTB8C36_Camila%20Silva%20Henriqu.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%202/crlv%20terceiro_Camila%20Silva%20Henriqu.jpeg</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20TERCEIRO/crlv%20terceiro._Camila%20Silva%20Henriqu.jpeg</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/f3.1_Camila%20Silva%20Henriqu.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/f3.2_Camila%20Silva%20Henriqu.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/f3_Camila%20Silva%20Henriqu.jpeg</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-16%20at%2019.10.10%20(2)_Camila%20Silva%20Henriqu.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-24%20at%2020.23.10_Camila%20Silva%20Henriqu.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-24%20at%2020.25.09_Camila%20Silva%20Henriqu.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-24%20at%2020.25.24_Camila%20Silva%20Henriqu.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-24%20at%2020.25.43_Camila%20Silva%20Henriqu.jpeg</t>
   </si>
   <si>
     <t>Valores</t>
@@ -5895,7 +5946,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72D61D6F-73C6-415B-9A64-53639FBBB1D8}" name="Tabela dinâmica1" cacheId="77" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72D61D6F-73C6-415B-9A64-53639FBBB1D8}" name="Tabela dinâmica1" cacheId="188" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:I8" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="48">
     <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
@@ -6036,8 +6087,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:AY73" headerRowDxfId="53" dataDxfId="52" totalsRowDxfId="51">
-  <autoFilter ref="A1:AY73" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:AY74" headerRowDxfId="53" dataDxfId="52" totalsRowDxfId="51">
+  <autoFilter ref="A1:AY74" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="51">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" totalsRowLabel="Total" dataDxfId="50">
       <extLst>
@@ -6388,7 +6439,7 @@
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{839C7E11-91E4-4DBD-9C5D-0DEA604FA9AC}">
-      <xlmsforms:msForm id="--soOq0dkkmCvV864R49jTu3qwhCFQBElTcewqtXSeRUQTE2N0tGUjlEMjREQU5OUzFKN1NSR1pQWS4u" isFormConnected="1" maxResponseId="82" latestEventMarker="149">
+      <xlmsforms:msForm id="--soOq0dkkmCvV864R49jTu3qwhCFQBElTcewqtXSeRUQTE2N0tGUjlEMjREQU5OUzFKN1NSR1pQWS4u" isFormConnected="1" maxResponseId="83" latestEventMarker="150">
         <xlmsforms:syncedQuestionId>id</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>startDate</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>submitDate</xlmsforms:syncedQuestionId>
@@ -6772,7 +6823,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CA122"/>
+  <dimension ref="A1:CA123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.85546875" style="14" hidden="1" customWidth="1"/>
@@ -16657,7 +16708,7 @@
         <v>82</v>
       </c>
       <c r="B73" s="12" t="s">
-        <v>1265</v>
+        <v>154</v>
       </c>
       <c r="C73" s="13"/>
       <c r="D73" s="13" t="s">
@@ -16791,55 +16842,113 @@
       <c r="BX73" s="12"/>
     </row>
     <row r="74" spans="1:76">
-      <c r="A74" s="5"/>
+      <c r="A74" s="5">
+        <v>83</v>
+      </c>
       <c r="B74" s="12"/>
-      <c r="C74" s="12"/>
-      <c r="D74" s="13"/>
-      <c r="E74" s="15"/>
-      <c r="F74" s="13"/>
-      <c r="G74" s="13"/>
-      <c r="H74" s="13"/>
-      <c r="I74" s="13"/>
-      <c r="J74" s="13"/>
-      <c r="K74" s="13"/>
-      <c r="L74" s="13"/>
-      <c r="M74" s="13"/>
-      <c r="N74" s="13"/>
-      <c r="O74" s="19"/>
-      <c r="P74" s="13"/>
-      <c r="Q74" s="16"/>
-      <c r="R74" s="12"/>
+      <c r="C74" s="13"/>
+      <c r="D74" s="13" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E74" s="15">
+        <v>46281</v>
+      </c>
+      <c r="F74" s="13" t="s">
+        <v>1380</v>
+      </c>
+      <c r="G74" s="13" t="s">
+        <v>1381</v>
+      </c>
+      <c r="H74" s="13" t="s">
+        <v>336</v>
+      </c>
+      <c r="I74" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="J74" s="13" t="s">
+        <v>1382</v>
+      </c>
+      <c r="K74" s="13" t="s">
+        <v>1383</v>
+      </c>
+      <c r="L74" s="13" t="s">
+        <v>1249</v>
+      </c>
+      <c r="M74" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="N74" s="13" t="s">
+        <v>1384</v>
+      </c>
+      <c r="O74" s="19" t="s">
+        <v>1385</v>
+      </c>
+      <c r="P74" s="13" t="s">
+        <v>1386</v>
+      </c>
+      <c r="Q74" s="16">
+        <v>46290.291701388902</v>
+      </c>
+      <c r="R74" s="12" t="s">
+        <v>155</v>
+      </c>
       <c r="S74" s="12"/>
       <c r="T74" s="12"/>
-      <c r="U74" s="17"/>
-      <c r="V74" s="20"/>
-      <c r="W74" s="13"/>
-      <c r="X74" s="13"/>
-      <c r="Y74" s="13"/>
+      <c r="U74" s="17">
+        <v>46290.297175925902</v>
+      </c>
+      <c r="V74" s="20" t="s">
+        <v>1253</v>
+      </c>
+      <c r="W74" s="13" t="s">
+        <v>1387</v>
+      </c>
+      <c r="X74" s="13" t="s">
+        <v>1255</v>
+      </c>
+      <c r="Y74" s="13" t="s">
+        <v>1388</v>
+      </c>
       <c r="Z74" s="12"/>
       <c r="AA74" s="13"/>
-      <c r="AB74" s="13"/>
+      <c r="AB74" s="13" t="s">
+        <v>1389</v>
+      </c>
       <c r="AC74" s="12"/>
       <c r="AD74" s="13"/>
-      <c r="AE74" s="13"/>
+      <c r="AE74" s="13" t="s">
+        <v>1390</v>
+      </c>
       <c r="AF74" s="12"/>
       <c r="AG74" s="13"/>
-      <c r="AH74" s="13"/>
+      <c r="AH74" s="13" t="s">
+        <v>1391</v>
+      </c>
       <c r="AI74" s="12"/>
       <c r="AJ74" s="13"/>
-      <c r="AK74" s="13"/>
+      <c r="AK74" s="13" t="s">
+        <v>1392</v>
+      </c>
       <c r="AL74" s="12"/>
       <c r="AM74" s="13"/>
-      <c r="AN74" s="13"/>
+      <c r="AN74" s="13" t="s">
+        <v>1393</v>
+      </c>
       <c r="AO74" s="12"/>
       <c r="AP74" s="13"/>
-      <c r="AQ74" s="13"/>
+      <c r="AQ74" s="13" t="s">
+        <v>1394</v>
+      </c>
       <c r="AR74" s="12"/>
       <c r="AS74" s="13"/>
-      <c r="AT74" s="13"/>
+      <c r="AT74" s="13" t="s">
+        <v>1395</v>
+      </c>
       <c r="AU74" s="12"/>
       <c r="AV74" s="13"/>
-      <c r="AW74" s="13"/>
+      <c r="AW74" s="13" t="s">
+        <v>1396</v>
+      </c>
       <c r="AX74" s="12"/>
       <c r="AY74" s="13"/>
     </row>
@@ -17321,56 +17430,57 @@
       <c r="AY83" s="13"/>
     </row>
     <row r="84" spans="1:51">
+      <c r="A84" s="5"/>
       <c r="B84" s="12"/>
       <c r="C84" s="12"/>
-      <c r="D84" s="12"/>
-      <c r="E84" s="17"/>
-      <c r="F84" s="12"/>
-      <c r="G84" s="12"/>
-      <c r="H84" s="12"/>
-      <c r="I84" s="12"/>
-      <c r="J84" s="12"/>
-      <c r="K84" s="12"/>
-      <c r="L84" s="12"/>
-      <c r="M84" s="12"/>
-      <c r="N84" s="12"/>
-      <c r="O84" s="12"/>
-      <c r="P84" s="12"/>
-      <c r="Q84" s="12"/>
-      <c r="R84" s="17"/>
+      <c r="D84" s="13"/>
+      <c r="E84" s="15"/>
+      <c r="F84" s="13"/>
+      <c r="G84" s="13"/>
+      <c r="H84" s="13"/>
+      <c r="I84" s="13"/>
+      <c r="J84" s="13"/>
+      <c r="K84" s="13"/>
+      <c r="L84" s="13"/>
+      <c r="M84" s="13"/>
+      <c r="N84" s="13"/>
+      <c r="O84" s="19"/>
+      <c r="P84" s="13"/>
+      <c r="Q84" s="16"/>
+      <c r="R84" s="12"/>
       <c r="S84" s="12"/>
       <c r="T84" s="12"/>
-      <c r="U84" s="12"/>
-      <c r="V84" s="12"/>
-      <c r="W84" s="12"/>
-      <c r="X84" s="12"/>
-      <c r="Y84" s="12"/>
+      <c r="U84" s="17"/>
+      <c r="V84" s="20"/>
+      <c r="W84" s="13"/>
+      <c r="X84" s="13"/>
+      <c r="Y84" s="13"/>
       <c r="Z84" s="12"/>
-      <c r="AA84" s="12"/>
-      <c r="AB84" s="12"/>
+      <c r="AA84" s="13"/>
+      <c r="AB84" s="13"/>
       <c r="AC84" s="12"/>
-      <c r="AD84" s="12"/>
-      <c r="AE84" s="12"/>
+      <c r="AD84" s="13"/>
+      <c r="AE84" s="13"/>
       <c r="AF84" s="12"/>
-      <c r="AG84" s="12"/>
-      <c r="AH84" s="12"/>
+      <c r="AG84" s="13"/>
+      <c r="AH84" s="13"/>
       <c r="AI84" s="12"/>
-      <c r="AJ84" s="12"/>
-      <c r="AK84" s="12"/>
+      <c r="AJ84" s="13"/>
+      <c r="AK84" s="13"/>
       <c r="AL84" s="12"/>
-      <c r="AM84" s="12"/>
-      <c r="AN84" s="12"/>
+      <c r="AM84" s="13"/>
+      <c r="AN84" s="13"/>
       <c r="AO84" s="12"/>
-      <c r="AP84" s="12"/>
-      <c r="AQ84" s="12"/>
+      <c r="AP84" s="13"/>
+      <c r="AQ84" s="13"/>
       <c r="AR84" s="12"/>
-      <c r="AS84" s="12"/>
-      <c r="AT84" s="12"/>
+      <c r="AS84" s="13"/>
+      <c r="AT84" s="13"/>
       <c r="AU84" s="12"/>
-      <c r="AV84" s="12"/>
-      <c r="AW84" s="12"/>
+      <c r="AV84" s="13"/>
+      <c r="AW84" s="13"/>
       <c r="AX84" s="12"/>
-      <c r="AY84" s="12"/>
+      <c r="AY84" s="13"/>
     </row>
     <row r="85" spans="1:51">
       <c r="B85" s="12"/>
@@ -19348,9 +19458,61 @@
       <c r="AX122" s="12"/>
       <c r="AY122" s="12"/>
     </row>
+    <row r="123" spans="2:51">
+      <c r="B123" s="12"/>
+      <c r="C123" s="12"/>
+      <c r="D123" s="12"/>
+      <c r="E123" s="17"/>
+      <c r="F123" s="12"/>
+      <c r="G123" s="12"/>
+      <c r="H123" s="12"/>
+      <c r="I123" s="12"/>
+      <c r="J123" s="12"/>
+      <c r="K123" s="12"/>
+      <c r="L123" s="12"/>
+      <c r="M123" s="12"/>
+      <c r="N123" s="12"/>
+      <c r="O123" s="12"/>
+      <c r="P123" s="12"/>
+      <c r="Q123" s="12"/>
+      <c r="R123" s="17"/>
+      <c r="S123" s="12"/>
+      <c r="T123" s="12"/>
+      <c r="U123" s="12"/>
+      <c r="V123" s="12"/>
+      <c r="W123" s="12"/>
+      <c r="X123" s="12"/>
+      <c r="Y123" s="12"/>
+      <c r="Z123" s="12"/>
+      <c r="AA123" s="12"/>
+      <c r="AB123" s="12"/>
+      <c r="AC123" s="12"/>
+      <c r="AD123" s="12"/>
+      <c r="AE123" s="12"/>
+      <c r="AF123" s="12"/>
+      <c r="AG123" s="12"/>
+      <c r="AH123" s="12"/>
+      <c r="AI123" s="12"/>
+      <c r="AJ123" s="12"/>
+      <c r="AK123" s="12"/>
+      <c r="AL123" s="12"/>
+      <c r="AM123" s="12"/>
+      <c r="AN123" s="12"/>
+      <c r="AO123" s="12"/>
+      <c r="AP123" s="12"/>
+      <c r="AQ123" s="12"/>
+      <c r="AR123" s="12"/>
+      <c r="AS123" s="12"/>
+      <c r="AT123" s="12"/>
+      <c r="AU123" s="12"/>
+      <c r="AV123" s="12"/>
+      <c r="AW123" s="12"/>
+      <c r="AX123" s="12"/>
+      <c r="AY123" s="12"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B73" xr:uid="{7B0F8D9B-CAD7-43B9-9768-9C793FE51B76}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B74" xr:uid="{7B0F8D9B-CAD7-43B9-9768-9C793FE51B76}">
       <formula1>"CONCLUÍDO, DOCUMENTO PENDENTE, ENVIADO PARA SEGURADORA,  FINALIZADO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -19391,7 +19553,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>1380</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -19405,33 +19567,33 @@
         <v>136</v>
       </c>
       <c r="H4" t="s">
-        <v>1381</v>
+        <v>1398</v>
       </c>
       <c r="I4" t="s">
-        <v>1382</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="11" t="s">
-        <v>1383</v>
+        <v>1400</v>
       </c>
       <c r="B5" t="s">
-        <v>1384</v>
+        <v>1401</v>
       </c>
       <c r="C5" t="s">
-        <v>1385</v>
+        <v>1402</v>
       </c>
       <c r="D5" t="s">
-        <v>1384</v>
+        <v>1401</v>
       </c>
       <c r="E5" t="s">
-        <v>1385</v>
+        <v>1402</v>
       </c>
       <c r="F5" t="s">
-        <v>1384</v>
+        <v>1401</v>
       </c>
       <c r="G5" t="s">
-        <v>1385</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -19488,7 +19650,7 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>1386</v>
+        <v>1403</v>
       </c>
       <c r="B8">
         <v>1</v>

</xml_diff>

<commit_message>
feat: improve fleet sync and email resolution logic
- Integrate Supabase client in the server for persistent operations
- Add intelligent base/filial normalization for automated email routing
- Update Google Sheets sync to preserve existing local vehicle data
- Enhance UI with additional icons and UI/UX improvements in ConfigPage
</commit_message>
<xml_diff>
--- a/data/Comunicado de Sinistro_Frota Pesada.xlsx
+++ b/data/Comunicado de Sinistro_Frota Pesada.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30524"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="519" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE2DE28-8AC7-4A85-AE1E-89255EACDEF1}"/>
+  <xr:revisionPtr revIDLastSave="524" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15D3009F-6172-4D6D-B1D2-2EF4325260D6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="188" r:id="rId3"/>
+    <pivotCache cacheId="386" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1898" uniqueCount="1404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="1420">
   <si>
     <t>Id</t>
   </si>
@@ -4239,6 +4239,54 @@
   </si>
   <si>
     <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-16%20at%2019.10.10%20(2)_Camila%20Silva%20Henriqu.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-24%20at%2020.23.10_Camila%20Silva%20Henriqu.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-24%20at%2020.25.09_Camila%20Silva%20Henriqu.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-24%20at%2020.25.24_Camila%20Silva%20Henriqu.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-24%20at%2020.25.43_Camila%20Silva%20Henriqu.jpeg</t>
+  </si>
+  <si>
+    <t>17:10</t>
+  </si>
+  <si>
+    <t>AVENIDA ENGENHEIRO AUGUSTO BARATA, SABOÓ</t>
+  </si>
+  <si>
+    <t>RNL4D77</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EVERTON OLÍMPIO </t>
+  </si>
+  <si>
+    <t>NÃO INFORMADO</t>
+  </si>
+  <si>
+    <t>GYS3A17</t>
+  </si>
+  <si>
+    <t>QUANDO PARADO NA VIA INFORMADA, TIVE QUE DAR RÉ, PARA UM VEÍCULO EFETUAR A CONVERÇÃO. QUANDO DANDO RÉ, ENCOSTEI NO CAMINHÃO QUE ESTAVA ATRÁS, OCASIONANDO UM PEQUENO DANO NO PARA-CHOQUE DO MESMO.</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/Pergunta/AVISO%20DE%20SINISTRO_Paulo%20Alves%20Pereira%206.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/AVISO%20DE%20SINISTRO/REGISTRO%20DE%20OCORR%C3%8ANCIA_Paulo%20Alves%20Pereira%206.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA/BOLETIM%20DE%20OCORR%C3%8ANCIA_Paulo%20Alves%20Pereira%202.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DECLARA%C3%87%C3%83O%20DE%20PR%C3%93PRIO%20PUNHO/CNH_THIAGO_EUZEBIO_Paulo%20Alves%20Pereira%201.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/CNH%20MOTORISTA%20RISEL/CRLV%20%20%2031.10.2026_Paulo%20Alves%20Pereira.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/_layouts/15/Doc.aspx?sourcedoc=%7B2BB2054F-F177-4BEC-BCC8-C50FE237D3FF%7D&amp;file=documento_Paulo%20Alves%20Pereira.docx&amp;action=default&amp;mobileredirect=true</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/_layouts/15/Doc.aspx?sourcedoc=%7B45641B1E-BDEB-43D6-B2B1-DF29D97C946F%7D&amp;file=documento_Paulo%20Alves%20Pereira.docx&amp;action=default&amp;mobileredirect=true</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-28%20at%2009.56.38%20(1)_Paulo%20Alves%20Pereira.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-28%20at%2009.56.38_Paulo%20Alves%20Pereira.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-28%20at%2009.56.39%20(1)_Paulo%20Alves%20Pereira.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-28%20at%2009.56.39_Paulo%20Alves%20Pereira.jpeg</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-28%20at%2011.09.43%20(1)_Paulo%20Alves%20Pereira.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-28%20at%2011.09.43%20(2)_Paulo%20Alves%20Pereira.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-28%20at%2011.09.43_Paulo%20Alves%20Pereira.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-28%20at%2011.09.44_Paulo%20Alves%20Pereira.jpeg</t>
   </si>
   <si>
     <t>Valores</t>
@@ -4346,7 +4394,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -4416,6 +4464,12 @@
     </xf>
     <xf numFmtId="22" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5946,7 +6000,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72D61D6F-73C6-415B-9A64-53639FBBB1D8}" name="Tabela dinâmica1" cacheId="188" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72D61D6F-73C6-415B-9A64-53639FBBB1D8}" name="Tabela dinâmica1" cacheId="386" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:I8" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="48">
     <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
@@ -6087,8 +6141,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:AY74" headerRowDxfId="53" dataDxfId="52" totalsRowDxfId="51">
-  <autoFilter ref="A1:AY74" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:AY75" headerRowDxfId="53" dataDxfId="52" totalsRowDxfId="51">
+  <autoFilter ref="A1:AY75" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="51">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" totalsRowLabel="Total" dataDxfId="50">
       <extLst>
@@ -6439,7 +6493,7 @@
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{839C7E11-91E4-4DBD-9C5D-0DEA604FA9AC}">
-      <xlmsforms:msForm id="--soOq0dkkmCvV864R49jTu3qwhCFQBElTcewqtXSeRUQTE2N0tGUjlEMjREQU5OUzFKN1NSR1pQWS4u" isFormConnected="1" maxResponseId="83" latestEventMarker="150">
+      <xlmsforms:msForm id="--soOq0dkkmCvV864R49jTu3qwhCFQBElTcewqtXSeRUQTE2N0tGUjlEMjREQU5OUzFKN1NSR1pQWS4u" isFormConnected="1" maxResponseId="84" latestEventMarker="151">
         <xlmsforms:syncedQuestionId>id</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>startDate</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>submitDate</xlmsforms:syncedQuestionId>
@@ -6823,7 +6877,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CA123"/>
+  <dimension ref="A1:CA124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.85546875" style="14" hidden="1" customWidth="1"/>
@@ -16953,56 +17007,114 @@
       <c r="AY74" s="13"/>
     </row>
     <row r="75" spans="1:76">
-      <c r="A75" s="5"/>
+      <c r="A75" s="26">
+        <v>84</v>
+      </c>
       <c r="B75" s="12"/>
-      <c r="C75" s="12"/>
-      <c r="D75" s="13"/>
-      <c r="E75" s="15"/>
-      <c r="F75" s="13"/>
-      <c r="G75" s="13"/>
-      <c r="H75" s="13"/>
-      <c r="I75" s="13"/>
-      <c r="J75" s="13"/>
-      <c r="K75" s="13"/>
-      <c r="L75" s="13"/>
-      <c r="M75" s="13"/>
-      <c r="N75" s="13"/>
-      <c r="O75" s="19"/>
-      <c r="P75" s="13"/>
-      <c r="Q75" s="16"/>
-      <c r="R75" s="12"/>
-      <c r="S75" s="12"/>
-      <c r="T75" s="12"/>
-      <c r="U75" s="17"/>
-      <c r="V75" s="20"/>
-      <c r="W75" s="13"/>
-      <c r="X75" s="13"/>
-      <c r="Y75" s="13"/>
-      <c r="Z75" s="12"/>
+      <c r="C75" s="13"/>
+      <c r="D75" s="13" t="s">
+        <v>1363</v>
+      </c>
+      <c r="E75" s="15">
+        <v>46289</v>
+      </c>
+      <c r="F75" s="13" t="s">
+        <v>1397</v>
+      </c>
+      <c r="G75" s="13" t="s">
+        <v>1398</v>
+      </c>
+      <c r="H75" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="I75" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="J75" s="13" t="s">
+        <v>1399</v>
+      </c>
+      <c r="K75" s="13" t="s">
+        <v>1029</v>
+      </c>
+      <c r="L75" s="13" t="s">
+        <v>1400</v>
+      </c>
+      <c r="M75" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N75" s="13" t="s">
+        <v>1401</v>
+      </c>
+      <c r="O75" s="19" t="s">
+        <v>1401</v>
+      </c>
+      <c r="P75" s="13" t="s">
+        <v>1402</v>
+      </c>
+      <c r="Q75" s="16">
+        <v>46294.493055555598</v>
+      </c>
+      <c r="R75" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="S75" s="27"/>
+      <c r="T75" s="27"/>
+      <c r="U75" s="17">
+        <v>46294.501157407401</v>
+      </c>
+      <c r="V75" s="20" t="s">
+        <v>1368</v>
+      </c>
+      <c r="W75" s="13" t="s">
+        <v>1403</v>
+      </c>
+      <c r="X75" s="13" t="s">
+        <v>1370</v>
+      </c>
+      <c r="Y75" s="13" t="s">
+        <v>1404</v>
+      </c>
+      <c r="Z75" s="27"/>
       <c r="AA75" s="13"/>
-      <c r="AB75" s="13"/>
-      <c r="AC75" s="12"/>
+      <c r="AB75" s="13" t="s">
+        <v>1405</v>
+      </c>
+      <c r="AC75" s="27"/>
       <c r="AD75" s="13"/>
-      <c r="AE75" s="13"/>
-      <c r="AF75" s="12"/>
+      <c r="AE75" s="13" t="s">
+        <v>1406</v>
+      </c>
+      <c r="AF75" s="27"/>
       <c r="AG75" s="13"/>
-      <c r="AH75" s="13"/>
-      <c r="AI75" s="12"/>
+      <c r="AH75" s="13" t="s">
+        <v>1407</v>
+      </c>
+      <c r="AI75" s="27"/>
       <c r="AJ75" s="13"/>
-      <c r="AK75" s="13"/>
-      <c r="AL75" s="12"/>
+      <c r="AK75" s="13" t="s">
+        <v>1408</v>
+      </c>
+      <c r="AL75" s="27"/>
       <c r="AM75" s="13"/>
-      <c r="AN75" s="13"/>
-      <c r="AO75" s="12"/>
+      <c r="AN75" s="13" t="s">
+        <v>1409</v>
+      </c>
+      <c r="AO75" s="27"/>
       <c r="AP75" s="13"/>
-      <c r="AQ75" s="13"/>
-      <c r="AR75" s="12"/>
+      <c r="AQ75" s="13" t="s">
+        <v>1410</v>
+      </c>
+      <c r="AR75" s="27"/>
       <c r="AS75" s="13"/>
-      <c r="AT75" s="13"/>
-      <c r="AU75" s="12"/>
+      <c r="AT75" s="13" t="s">
+        <v>1411</v>
+      </c>
+      <c r="AU75" s="27"/>
       <c r="AV75" s="13"/>
-      <c r="AW75" s="13"/>
-      <c r="AX75" s="12"/>
+      <c r="AW75" s="13" t="s">
+        <v>1412</v>
+      </c>
+      <c r="AX75" s="27"/>
       <c r="AY75" s="13"/>
     </row>
     <row r="76" spans="1:76">
@@ -17483,56 +17595,57 @@
       <c r="AY84" s="13"/>
     </row>
     <row r="85" spans="1:51">
+      <c r="A85" s="5"/>
       <c r="B85" s="12"/>
       <c r="C85" s="12"/>
-      <c r="D85" s="12"/>
-      <c r="E85" s="17"/>
-      <c r="F85" s="12"/>
-      <c r="G85" s="12"/>
-      <c r="H85" s="12"/>
-      <c r="I85" s="12"/>
-      <c r="J85" s="12"/>
-      <c r="K85" s="12"/>
-      <c r="L85" s="12"/>
-      <c r="M85" s="12"/>
-      <c r="N85" s="12"/>
-      <c r="O85" s="12"/>
-      <c r="P85" s="12"/>
-      <c r="Q85" s="12"/>
-      <c r="R85" s="17"/>
+      <c r="D85" s="13"/>
+      <c r="E85" s="15"/>
+      <c r="F85" s="13"/>
+      <c r="G85" s="13"/>
+      <c r="H85" s="13"/>
+      <c r="I85" s="13"/>
+      <c r="J85" s="13"/>
+      <c r="K85" s="13"/>
+      <c r="L85" s="13"/>
+      <c r="M85" s="13"/>
+      <c r="N85" s="13"/>
+      <c r="O85" s="19"/>
+      <c r="P85" s="13"/>
+      <c r="Q85" s="16"/>
+      <c r="R85" s="12"/>
       <c r="S85" s="12"/>
       <c r="T85" s="12"/>
-      <c r="U85" s="12"/>
-      <c r="V85" s="12"/>
-      <c r="W85" s="12"/>
-      <c r="X85" s="12"/>
-      <c r="Y85" s="12"/>
+      <c r="U85" s="17"/>
+      <c r="V85" s="20"/>
+      <c r="W85" s="13"/>
+      <c r="X85" s="13"/>
+      <c r="Y85" s="13"/>
       <c r="Z85" s="12"/>
-      <c r="AA85" s="12"/>
-      <c r="AB85" s="12"/>
+      <c r="AA85" s="13"/>
+      <c r="AB85" s="13"/>
       <c r="AC85" s="12"/>
-      <c r="AD85" s="12"/>
-      <c r="AE85" s="12"/>
+      <c r="AD85" s="13"/>
+      <c r="AE85" s="13"/>
       <c r="AF85" s="12"/>
-      <c r="AG85" s="12"/>
-      <c r="AH85" s="12"/>
+      <c r="AG85" s="13"/>
+      <c r="AH85" s="13"/>
       <c r="AI85" s="12"/>
-      <c r="AJ85" s="12"/>
-      <c r="AK85" s="12"/>
+      <c r="AJ85" s="13"/>
+      <c r="AK85" s="13"/>
       <c r="AL85" s="12"/>
-      <c r="AM85" s="12"/>
-      <c r="AN85" s="12"/>
+      <c r="AM85" s="13"/>
+      <c r="AN85" s="13"/>
       <c r="AO85" s="12"/>
-      <c r="AP85" s="12"/>
-      <c r="AQ85" s="12"/>
+      <c r="AP85" s="13"/>
+      <c r="AQ85" s="13"/>
       <c r="AR85" s="12"/>
-      <c r="AS85" s="12"/>
-      <c r="AT85" s="12"/>
+      <c r="AS85" s="13"/>
+      <c r="AT85" s="13"/>
       <c r="AU85" s="12"/>
-      <c r="AV85" s="12"/>
-      <c r="AW85" s="12"/>
+      <c r="AV85" s="13"/>
+      <c r="AW85" s="13"/>
       <c r="AX85" s="12"/>
-      <c r="AY85" s="12"/>
+      <c r="AY85" s="13"/>
     </row>
     <row r="86" spans="1:51">
       <c r="B86" s="12"/>
@@ -19510,9 +19623,61 @@
       <c r="AX123" s="12"/>
       <c r="AY123" s="12"/>
     </row>
+    <row r="124" spans="2:51">
+      <c r="B124" s="12"/>
+      <c r="C124" s="12"/>
+      <c r="D124" s="12"/>
+      <c r="E124" s="17"/>
+      <c r="F124" s="12"/>
+      <c r="G124" s="12"/>
+      <c r="H124" s="12"/>
+      <c r="I124" s="12"/>
+      <c r="J124" s="12"/>
+      <c r="K124" s="12"/>
+      <c r="L124" s="12"/>
+      <c r="M124" s="12"/>
+      <c r="N124" s="12"/>
+      <c r="O124" s="12"/>
+      <c r="P124" s="12"/>
+      <c r="Q124" s="12"/>
+      <c r="R124" s="17"/>
+      <c r="S124" s="12"/>
+      <c r="T124" s="12"/>
+      <c r="U124" s="12"/>
+      <c r="V124" s="12"/>
+      <c r="W124" s="12"/>
+      <c r="X124" s="12"/>
+      <c r="Y124" s="12"/>
+      <c r="Z124" s="12"/>
+      <c r="AA124" s="12"/>
+      <c r="AB124" s="12"/>
+      <c r="AC124" s="12"/>
+      <c r="AD124" s="12"/>
+      <c r="AE124" s="12"/>
+      <c r="AF124" s="12"/>
+      <c r="AG124" s="12"/>
+      <c r="AH124" s="12"/>
+      <c r="AI124" s="12"/>
+      <c r="AJ124" s="12"/>
+      <c r="AK124" s="12"/>
+      <c r="AL124" s="12"/>
+      <c r="AM124" s="12"/>
+      <c r="AN124" s="12"/>
+      <c r="AO124" s="12"/>
+      <c r="AP124" s="12"/>
+      <c r="AQ124" s="12"/>
+      <c r="AR124" s="12"/>
+      <c r="AS124" s="12"/>
+      <c r="AT124" s="12"/>
+      <c r="AU124" s="12"/>
+      <c r="AV124" s="12"/>
+      <c r="AW124" s="12"/>
+      <c r="AX124" s="12"/>
+      <c r="AY124" s="12"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B74" xr:uid="{7B0F8D9B-CAD7-43B9-9768-9C793FE51B76}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B75" xr:uid="{7B0F8D9B-CAD7-43B9-9768-9C793FE51B76}">
       <formula1>"CONCLUÍDO, DOCUMENTO PENDENTE, ENVIADO PARA SEGURADORA,  FINALIZADO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -19553,7 +19718,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>1397</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -19567,33 +19732,33 @@
         <v>136</v>
       </c>
       <c r="H4" t="s">
-        <v>1398</v>
+        <v>1414</v>
       </c>
       <c r="I4" t="s">
-        <v>1399</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="11" t="s">
-        <v>1400</v>
+        <v>1416</v>
       </c>
       <c r="B5" t="s">
-        <v>1401</v>
+        <v>1417</v>
       </c>
       <c r="C5" t="s">
-        <v>1402</v>
+        <v>1418</v>
       </c>
       <c r="D5" t="s">
-        <v>1401</v>
+        <v>1417</v>
       </c>
       <c r="E5" t="s">
-        <v>1402</v>
+        <v>1418</v>
       </c>
       <c r="F5" t="s">
-        <v>1401</v>
+        <v>1417</v>
       </c>
       <c r="G5" t="s">
-        <v>1402</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -19650,7 +19815,7 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>1403</v>
+        <v>1419</v>
       </c>
       <c r="B8">
         <v>1</v>

</xml_diff>

<commit_message>
feat(sinistros): update registry and improve reservation emails
- Add new incident record (SIN-85) to database
- Update reservation approval email template with clear return instructions
- Prepare UserDailyUseForm for URL-based state management
</commit_message>
<xml_diff>
--- a/data/Comunicado de Sinistro_Frota Pesada.xlsx
+++ b/data/Comunicado de Sinistro_Frota Pesada.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30524"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="524" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15D3009F-6172-4D6D-B1D2-2EF4325260D6}"/>
+  <xr:revisionPtr revIDLastSave="528" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A14A625-0FC0-469E-B7D7-688FD3EF1CB7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="386" r:id="rId3"/>
+    <pivotCache cacheId="264" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="1420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1948" uniqueCount="1441">
   <si>
     <t>Id</t>
   </si>
@@ -4287,6 +4287,69 @@
   </si>
   <si>
     <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-28%20at%2011.09.43%20(1)_Paulo%20Alves%20Pereira.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-28%20at%2011.09.43%20(2)_Paulo%20Alves%20Pereira.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-28%20at%2011.09.43_Paulo%20Alves%20Pereira.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-09-28%20at%2011.09.44_Paulo%20Alves%20Pereira.jpeg</t>
+  </si>
+  <si>
+    <t>Thiago Ferreira Lima</t>
+  </si>
+  <si>
+    <t>12:30</t>
+  </si>
+  <si>
+    <t>Restaurante Andorinha</t>
+  </si>
+  <si>
+    <t>Ribeirão Branco</t>
+  </si>
+  <si>
+    <t>END2537</t>
+  </si>
+  <si>
+    <t>PEDRO DA SILVA PRAXEDES</t>
+  </si>
+  <si>
+    <t>Priscila Carolina Mendes</t>
+  </si>
+  <si>
+    <t>VITOR VERGTZ SIVA</t>
+  </si>
+  <si>
+    <t>+55 42 9808-9498</t>
+  </si>
+  <si>
+    <t>166241</t>
+  </si>
+  <si>
+    <t>thiago.lima@risel.com.br</t>
+  </si>
+  <si>
+    <t>EU PEDRO ESTAVA COM O CAMINHÃO END2537  ESTACIONADO NO PATIO DO RESTAURANTE ANDORINHA, ALMOÇANDO, QUANDO AS VIATURAS MILITARES COMPOSTA POR TRÊS VEICULOS PARARAM NO RESTAURANTE, APÓS O HORARIO DE ALMOÇO AS VIATURAS FORAM SAIR DE TRÁS DO CAMINHÃO DA EMPRESA, UMA DELAS VEIO A COLIDIR NO PARACHOQUE TRASEIRO, OCOSIONANDO QUEBRA DO PARACHOQUE DIANTEIRO DA VIATURA MERCEDES BENZ 166241.</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/Pergunta/aviso%20de%20sinistro_Thiago%20Ferreira%20Lima.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/AVISO%20DE%20SINISTRO/REGISTRO%20DE%20OCORRENCIA%20-%20PEDRO%20PRAXEDES%20DA%20SI_Thiago%20Ferreira%20Lima.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA/BOLETIM%20PEDRO%20PRAXEDES_Thiago%20Ferreira%20Lima.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DECLARA%C3%87%C3%83O%20DE%20PR%C3%93PRIO%20PUNHO/CNH-e.pdf%20(3)_Thiago%20Ferreira%20Lima.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/CNH%20MOTORISTA%20RISEL/F-1140%20END2537_Thiago%20Ferreira%20Lima.pdf</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%202/WhatsApp%20Image%202026-10-02%20at%2010.10.26_Thiago%20Ferreira%20Lima.jpeg</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20TERCEIRO/WhatsApp%20Image%202026-10-02%20at%2010.10.01_Thiago%20Ferreira%20Lima.jpeg</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-22%20at%2013.37.58%20(2)_Thiago%20Ferreira%20Lima.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-22%20at%2013.37.58%20(1)_Thiago%20Ferreira%20Lima.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-22%20at%2013.37.58_Thiago%20Ferreira%20Lima.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-22%20at%2013.37.59%20(1)_Thiago%20Ferreira%20Lima.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-22%20at%2013.37.59_Thiago%20Ferreira%20Lima.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-22%20at%2013.59.43%20(1)_Thiago%20Ferreira%20Lima.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-22%20at%2013.59.43_Thiago%20Ferreira%20Lima.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-22%20at%2016.36.27_Thiago%20Ferreira%20Lima.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/DOCUMENTO%20DO%20VE%C3%8DCULO%20DA%20FROTA%201/WhatsApp%20Image%202026-09-22%20at%2016.36.28_Thiago%20Ferreira%20Lima.jpeg</t>
+  </si>
+  <si>
+    <t>https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-10-02%20at%2010.04.23%20(1)_Thiago%20Ferreira%20Lima.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-10-02%20at%2010.04.23_Thiago%20Ferreira%20Lima.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-10-02%20at%2010.04.22%20(1)_Thiago%20Ferreira%20Lima.jpeg; https://riselcombustiveis-my.sharepoint.com/personal/deny_goncalves_risel_com_br/Documents/Aplicativos/Microsoft%20Forms/Comunicado%20de%20Sinistro%20-%20Frota%20Pesada/FOTOS%20DO%20OCORRIDO/WhatsApp%20Image%202026-10-02%20at%2010.04.22_Thiago%20Ferreira%20Lima.jpeg</t>
   </si>
   <si>
     <t>Valores</t>
@@ -5590,6 +5653,9 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
       <x14:pivotCacheDefinition/>
     </ext>
+    <ext xmlns:xlpdsc="http://schemas.microsoft.com/office/spreadsheetml/2026/pivotDataSourceClean" uri="{F4336242-56EE-4DD3-A5F7-E900642BF6E9}">
+      <xlpdsc:dataSourceClean>1</xlpdsc:dataSourceClean>
+    </ext>
   </extLst>
 </pivotCacheDefinition>
 </file>
@@ -6000,7 +6066,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72D61D6F-73C6-415B-9A64-53639FBBB1D8}" name="Tabela dinâmica1" cacheId="386" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72D61D6F-73C6-415B-9A64-53639FBBB1D8}" name="Tabela dinâmica1" cacheId="264" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:I8" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="48">
     <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
@@ -6141,8 +6207,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:AY75" headerRowDxfId="53" dataDxfId="52" totalsRowDxfId="51">
-  <autoFilter ref="A1:AY75" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:AY76" headerRowDxfId="53" dataDxfId="52" totalsRowDxfId="51">
+  <autoFilter ref="A1:AY76" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="51">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" totalsRowLabel="Total" dataDxfId="50">
       <extLst>
@@ -6493,7 +6559,7 @@
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{839C7E11-91E4-4DBD-9C5D-0DEA604FA9AC}">
-      <xlmsforms:msForm id="--soOq0dkkmCvV864R49jTu3qwhCFQBElTcewqtXSeRUQTE2N0tGUjlEMjREQU5OUzFKN1NSR1pQWS4u" isFormConnected="1" maxResponseId="84" latestEventMarker="151">
+      <xlmsforms:msForm id="--soOq0dkkmCvV864R49jTu3qwhCFQBElTcewqtXSeRUQTE2N0tGUjlEMjREQU5OUzFKN1NSR1pQWS4u" isFormConnected="1" maxResponseId="85" latestEventMarker="152">
         <xlmsforms:syncedQuestionId>id</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>startDate</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>submitDate</xlmsforms:syncedQuestionId>
@@ -6877,11 +6943,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CA124"/>
+  <dimension ref="A1:CA125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.85546875" style="14" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="26" style="8" customWidth="1"/>
     <col min="3" max="3" width="15.140625" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.140625" style="14" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.140625" style="10" customWidth="1"/>
@@ -17007,7 +17073,7 @@
       <c r="AY74" s="13"/>
     </row>
     <row r="75" spans="1:76">
-      <c r="A75" s="26">
+      <c r="A75" s="5">
         <v>84</v>
       </c>
       <c r="B75" s="12"/>
@@ -17054,11 +17120,11 @@
       <c r="Q75" s="16">
         <v>46294.493055555598</v>
       </c>
-      <c r="R75" s="27" t="s">
+      <c r="R75" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="S75" s="27"/>
-      <c r="T75" s="27"/>
+      <c r="S75" s="12"/>
+      <c r="T75" s="12"/>
       <c r="U75" s="17">
         <v>46294.501157407401</v>
       </c>
@@ -17074,100 +17140,158 @@
       <c r="Y75" s="13" t="s">
         <v>1404</v>
       </c>
-      <c r="Z75" s="27"/>
+      <c r="Z75" s="12"/>
       <c r="AA75" s="13"/>
       <c r="AB75" s="13" t="s">
         <v>1405</v>
       </c>
-      <c r="AC75" s="27"/>
+      <c r="AC75" s="12"/>
       <c r="AD75" s="13"/>
       <c r="AE75" s="13" t="s">
         <v>1406</v>
       </c>
-      <c r="AF75" s="27"/>
+      <c r="AF75" s="12"/>
       <c r="AG75" s="13"/>
       <c r="AH75" s="13" t="s">
         <v>1407</v>
       </c>
-      <c r="AI75" s="27"/>
+      <c r="AI75" s="12"/>
       <c r="AJ75" s="13"/>
       <c r="AK75" s="13" t="s">
         <v>1408</v>
       </c>
-      <c r="AL75" s="27"/>
+      <c r="AL75" s="12"/>
       <c r="AM75" s="13"/>
       <c r="AN75" s="13" t="s">
         <v>1409</v>
       </c>
-      <c r="AO75" s="27"/>
+      <c r="AO75" s="12"/>
       <c r="AP75" s="13"/>
       <c r="AQ75" s="13" t="s">
         <v>1410</v>
       </c>
-      <c r="AR75" s="27"/>
+      <c r="AR75" s="12"/>
       <c r="AS75" s="13"/>
       <c r="AT75" s="13" t="s">
         <v>1411</v>
       </c>
-      <c r="AU75" s="27"/>
+      <c r="AU75" s="12"/>
       <c r="AV75" s="13"/>
       <c r="AW75" s="13" t="s">
         <v>1412</v>
       </c>
-      <c r="AX75" s="27"/>
+      <c r="AX75" s="12"/>
       <c r="AY75" s="13"/>
     </row>
     <row r="76" spans="1:76">
-      <c r="A76" s="5"/>
+      <c r="A76" s="26">
+        <v>85</v>
+      </c>
       <c r="B76" s="12"/>
-      <c r="C76" s="12"/>
-      <c r="D76" s="13"/>
-      <c r="E76" s="15"/>
-      <c r="F76" s="13"/>
-      <c r="G76" s="13"/>
-      <c r="H76" s="13"/>
-      <c r="I76" s="13"/>
-      <c r="J76" s="13"/>
-      <c r="K76" s="13"/>
-      <c r="L76" s="13"/>
-      <c r="M76" s="13"/>
-      <c r="N76" s="13"/>
-      <c r="O76" s="19"/>
-      <c r="P76" s="13"/>
-      <c r="Q76" s="16"/>
-      <c r="R76" s="12"/>
-      <c r="S76" s="12"/>
-      <c r="T76" s="12"/>
-      <c r="U76" s="17"/>
-      <c r="V76" s="20"/>
-      <c r="W76" s="13"/>
-      <c r="X76" s="13"/>
-      <c r="Y76" s="13"/>
-      <c r="Z76" s="12"/>
+      <c r="C76" s="13"/>
+      <c r="D76" s="13" t="s">
+        <v>1413</v>
+      </c>
+      <c r="E76" s="15">
+        <v>46287</v>
+      </c>
+      <c r="F76" s="13" t="s">
+        <v>1414</v>
+      </c>
+      <c r="G76" s="13" t="s">
+        <v>1415</v>
+      </c>
+      <c r="H76" s="13" t="s">
+        <v>1416</v>
+      </c>
+      <c r="I76" s="13" t="s">
+        <v>548</v>
+      </c>
+      <c r="J76" s="13" t="s">
+        <v>1417</v>
+      </c>
+      <c r="K76" s="13" t="s">
+        <v>1418</v>
+      </c>
+      <c r="L76" s="13" t="s">
+        <v>1419</v>
+      </c>
+      <c r="M76" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="N76" s="13" t="s">
+        <v>1420</v>
+      </c>
+      <c r="O76" s="19" t="s">
+        <v>1421</v>
+      </c>
+      <c r="P76" s="19" t="s">
+        <v>1422</v>
+      </c>
+      <c r="Q76" s="16">
+        <v>46297.4143287037</v>
+      </c>
+      <c r="R76" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="S76" s="27"/>
+      <c r="T76" s="27"/>
+      <c r="U76" s="17">
+        <v>46297.424826388902</v>
+      </c>
+      <c r="V76" s="20" t="s">
+        <v>1423</v>
+      </c>
+      <c r="W76" s="13" t="s">
+        <v>1424</v>
+      </c>
+      <c r="X76" s="13" t="s">
+        <v>1423</v>
+      </c>
+      <c r="Y76" s="13" t="s">
+        <v>1425</v>
+      </c>
+      <c r="Z76" s="27"/>
       <c r="AA76" s="13"/>
-      <c r="AB76" s="13"/>
-      <c r="AC76" s="12"/>
+      <c r="AB76" s="13" t="s">
+        <v>1426</v>
+      </c>
+      <c r="AC76" s="27"/>
       <c r="AD76" s="13"/>
-      <c r="AE76" s="13"/>
-      <c r="AF76" s="12"/>
+      <c r="AE76" s="13" t="s">
+        <v>1427</v>
+      </c>
+      <c r="AF76" s="27"/>
       <c r="AG76" s="13"/>
-      <c r="AH76" s="13"/>
-      <c r="AI76" s="12"/>
+      <c r="AH76" s="13" t="s">
+        <v>1428</v>
+      </c>
+      <c r="AI76" s="27"/>
       <c r="AJ76" s="13"/>
-      <c r="AK76" s="13"/>
-      <c r="AL76" s="12"/>
+      <c r="AK76" s="13" t="s">
+        <v>1429</v>
+      </c>
+      <c r="AL76" s="27"/>
       <c r="AM76" s="13"/>
-      <c r="AN76" s="13"/>
-      <c r="AO76" s="12"/>
+      <c r="AN76" s="13" t="s">
+        <v>1430</v>
+      </c>
+      <c r="AO76" s="27"/>
       <c r="AP76" s="13"/>
-      <c r="AQ76" s="13"/>
-      <c r="AR76" s="12"/>
+      <c r="AQ76" s="13" t="s">
+        <v>1431</v>
+      </c>
+      <c r="AR76" s="27"/>
       <c r="AS76" s="13"/>
-      <c r="AT76" s="13"/>
-      <c r="AU76" s="12"/>
+      <c r="AT76" s="13" t="s">
+        <v>1432</v>
+      </c>
+      <c r="AU76" s="27"/>
       <c r="AV76" s="13"/>
-      <c r="AW76" s="13"/>
-      <c r="AX76" s="12"/>
+      <c r="AW76" s="13" t="s">
+        <v>1433</v>
+      </c>
+      <c r="AX76" s="27"/>
       <c r="AY76" s="13"/>
     </row>
     <row r="77" spans="1:76">
@@ -17648,56 +17772,57 @@
       <c r="AY85" s="13"/>
     </row>
     <row r="86" spans="1:51">
+      <c r="A86" s="5"/>
       <c r="B86" s="12"/>
       <c r="C86" s="12"/>
-      <c r="D86" s="12"/>
-      <c r="E86" s="17"/>
-      <c r="F86" s="12"/>
-      <c r="G86" s="12"/>
-      <c r="H86" s="12"/>
-      <c r="I86" s="12"/>
-      <c r="J86" s="12"/>
-      <c r="K86" s="12"/>
-      <c r="L86" s="12"/>
-      <c r="M86" s="12"/>
-      <c r="N86" s="12"/>
-      <c r="O86" s="12"/>
-      <c r="P86" s="12"/>
-      <c r="Q86" s="12"/>
-      <c r="R86" s="17"/>
+      <c r="D86" s="13"/>
+      <c r="E86" s="15"/>
+      <c r="F86" s="13"/>
+      <c r="G86" s="13"/>
+      <c r="H86" s="13"/>
+      <c r="I86" s="13"/>
+      <c r="J86" s="13"/>
+      <c r="K86" s="13"/>
+      <c r="L86" s="13"/>
+      <c r="M86" s="13"/>
+      <c r="N86" s="13"/>
+      <c r="O86" s="19"/>
+      <c r="P86" s="13"/>
+      <c r="Q86" s="16"/>
+      <c r="R86" s="12"/>
       <c r="S86" s="12"/>
       <c r="T86" s="12"/>
-      <c r="U86" s="12"/>
-      <c r="V86" s="12"/>
-      <c r="W86" s="12"/>
-      <c r="X86" s="12"/>
-      <c r="Y86" s="12"/>
+      <c r="U86" s="17"/>
+      <c r="V86" s="20"/>
+      <c r="W86" s="13"/>
+      <c r="X86" s="13"/>
+      <c r="Y86" s="13"/>
       <c r="Z86" s="12"/>
-      <c r="AA86" s="12"/>
-      <c r="AB86" s="12"/>
+      <c r="AA86" s="13"/>
+      <c r="AB86" s="13"/>
       <c r="AC86" s="12"/>
-      <c r="AD86" s="12"/>
-      <c r="AE86" s="12"/>
+      <c r="AD86" s="13"/>
+      <c r="AE86" s="13"/>
       <c r="AF86" s="12"/>
-      <c r="AG86" s="12"/>
-      <c r="AH86" s="12"/>
+      <c r="AG86" s="13"/>
+      <c r="AH86" s="13"/>
       <c r="AI86" s="12"/>
-      <c r="AJ86" s="12"/>
-      <c r="AK86" s="12"/>
+      <c r="AJ86" s="13"/>
+      <c r="AK86" s="13"/>
       <c r="AL86" s="12"/>
-      <c r="AM86" s="12"/>
-      <c r="AN86" s="12"/>
+      <c r="AM86" s="13"/>
+      <c r="AN86" s="13"/>
       <c r="AO86" s="12"/>
-      <c r="AP86" s="12"/>
-      <c r="AQ86" s="12"/>
+      <c r="AP86" s="13"/>
+      <c r="AQ86" s="13"/>
       <c r="AR86" s="12"/>
-      <c r="AS86" s="12"/>
-      <c r="AT86" s="12"/>
+      <c r="AS86" s="13"/>
+      <c r="AT86" s="13"/>
       <c r="AU86" s="12"/>
-      <c r="AV86" s="12"/>
-      <c r="AW86" s="12"/>
+      <c r="AV86" s="13"/>
+      <c r="AW86" s="13"/>
       <c r="AX86" s="12"/>
-      <c r="AY86" s="12"/>
+      <c r="AY86" s="13"/>
     </row>
     <row r="87" spans="1:51">
       <c r="B87" s="12"/>
@@ -19675,9 +19800,61 @@
       <c r="AX124" s="12"/>
       <c r="AY124" s="12"/>
     </row>
+    <row r="125" spans="2:51">
+      <c r="B125" s="12"/>
+      <c r="C125" s="12"/>
+      <c r="D125" s="12"/>
+      <c r="E125" s="17"/>
+      <c r="F125" s="12"/>
+      <c r="G125" s="12"/>
+      <c r="H125" s="12"/>
+      <c r="I125" s="12"/>
+      <c r="J125" s="12"/>
+      <c r="K125" s="12"/>
+      <c r="L125" s="12"/>
+      <c r="M125" s="12"/>
+      <c r="N125" s="12"/>
+      <c r="O125" s="12"/>
+      <c r="P125" s="12"/>
+      <c r="Q125" s="12"/>
+      <c r="R125" s="17"/>
+      <c r="S125" s="12"/>
+      <c r="T125" s="12"/>
+      <c r="U125" s="12"/>
+      <c r="V125" s="12"/>
+      <c r="W125" s="12"/>
+      <c r="X125" s="12"/>
+      <c r="Y125" s="12"/>
+      <c r="Z125" s="12"/>
+      <c r="AA125" s="12"/>
+      <c r="AB125" s="12"/>
+      <c r="AC125" s="12"/>
+      <c r="AD125" s="12"/>
+      <c r="AE125" s="12"/>
+      <c r="AF125" s="12"/>
+      <c r="AG125" s="12"/>
+      <c r="AH125" s="12"/>
+      <c r="AI125" s="12"/>
+      <c r="AJ125" s="12"/>
+      <c r="AK125" s="12"/>
+      <c r="AL125" s="12"/>
+      <c r="AM125" s="12"/>
+      <c r="AN125" s="12"/>
+      <c r="AO125" s="12"/>
+      <c r="AP125" s="12"/>
+      <c r="AQ125" s="12"/>
+      <c r="AR125" s="12"/>
+      <c r="AS125" s="12"/>
+      <c r="AT125" s="12"/>
+      <c r="AU125" s="12"/>
+      <c r="AV125" s="12"/>
+      <c r="AW125" s="12"/>
+      <c r="AX125" s="12"/>
+      <c r="AY125" s="12"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B75" xr:uid="{7B0F8D9B-CAD7-43B9-9768-9C793FE51B76}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B76" xr:uid="{7B0F8D9B-CAD7-43B9-9768-9C793FE51B76}">
       <formula1>"CONCLUÍDO, DOCUMENTO PENDENTE, ENVIADO PARA SEGURADORA,  FINALIZADO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -19718,7 +19895,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>1413</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -19732,33 +19909,33 @@
         <v>136</v>
       </c>
       <c r="H4" t="s">
-        <v>1414</v>
+        <v>1435</v>
       </c>
       <c r="I4" t="s">
-        <v>1415</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="11" t="s">
-        <v>1416</v>
+        <v>1437</v>
       </c>
       <c r="B5" t="s">
-        <v>1417</v>
+        <v>1438</v>
       </c>
       <c r="C5" t="s">
-        <v>1418</v>
+        <v>1439</v>
       </c>
       <c r="D5" t="s">
-        <v>1417</v>
+        <v>1438</v>
       </c>
       <c r="E5" t="s">
-        <v>1418</v>
+        <v>1439</v>
       </c>
       <c r="F5" t="s">
-        <v>1417</v>
+        <v>1438</v>
       </c>
       <c r="G5" t="s">
-        <v>1418</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -19815,7 +19992,7 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>1419</v>
+        <v>1440</v>
       </c>
       <c r="B8">
         <v>1</v>

</xml_diff>